<commit_message>
added genes_additions to task 702
</commit_message>
<xml_diff>
--- a/Tasks/Task_702_TNFa_synthesis/genes_additions.xlsx
+++ b/Tasks/Task_702_TNFa_synthesis/genes_additions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26626"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Git\MSP_p3_2026_hormone_cytokine_task_creation\Current_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/juliawaldmeier/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{023EA2A3-F376-47B0-9891-F67FA55DF277}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CCB1693-FC33-6B46-AD18-3E0A356795A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{83A1BC92-ED54-4889-8F5C-FBE0ADADD62A}"/>
+    <workbookView xWindow="4440" yWindow="760" windowWidth="24960" windowHeight="17200" xr2:uid="{83A1BC92-ED54-4889-8F5C-FBE0ADADD62A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="154">
   <si>
     <t>MIRIAM</t>
   </si>
@@ -45,13 +45,466 @@
   </si>
   <si>
     <t>short_name</t>
+  </si>
+  <si>
+    <t>ENSG00000232810</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000232810</t>
+  </si>
+  <si>
+    <t>TNF</t>
+  </si>
+  <si>
+    <t>ENSG00000153037</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000153037</t>
+  </si>
+  <si>
+    <t>SRP54</t>
+  </si>
+  <si>
+    <t>SRP19</t>
+  </si>
+  <si>
+    <t>SRP68</t>
+  </si>
+  <si>
+    <t>ENSG00000167881</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000167881</t>
+  </si>
+  <si>
+    <t>SRP72</t>
+  </si>
+  <si>
+    <t>ENSG00000174780</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000174780</t>
+  </si>
+  <si>
+    <t>SRP14</t>
+  </si>
+  <si>
+    <t>ENSG00000140319</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000140319</t>
+  </si>
+  <si>
+    <t>SRP9</t>
+  </si>
+  <si>
+    <t>ENSG00000143742</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000143742</t>
+  </si>
+  <si>
+    <t>SRPRA</t>
+  </si>
+  <si>
+    <t>SRPRB</t>
+  </si>
+  <si>
+    <t>ENSG00000182934</t>
+  </si>
+  <si>
+    <t>ENSG00000144867</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000144867</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000182934</t>
+  </si>
+  <si>
+    <t>SEC61A1</t>
+  </si>
+  <si>
+    <t>SEC61A2</t>
+  </si>
+  <si>
+    <t>SEC61B</t>
+  </si>
+  <si>
+    <t>SEC61G</t>
+  </si>
+  <si>
+    <t>ENSG00000058262</t>
+  </si>
+  <si>
+    <t>ENSG00000065665</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000065665</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000058262</t>
+  </si>
+  <si>
+    <t>ENSG00000106803</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000106803</t>
+  </si>
+  <si>
+    <t>ENSG00000132432</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000132432</t>
+  </si>
+  <si>
+    <t>SPCS1</t>
+  </si>
+  <si>
+    <t>SPCS3</t>
+  </si>
+  <si>
+    <t>SPCS2</t>
+  </si>
+  <si>
+    <t>SEC11A</t>
+  </si>
+  <si>
+    <t>SEC11C</t>
+  </si>
+  <si>
+    <t>ENSG00000114902</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000114902</t>
+  </si>
+  <si>
+    <t>ENSG00000129128</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000129128</t>
+  </si>
+  <si>
+    <t>ENSG00000118363</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000118363</t>
+  </si>
+  <si>
+    <t>ENSG00000140612</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000140612</t>
+  </si>
+  <si>
+    <t>ENSG00000166562</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000166562</t>
+  </si>
+  <si>
+    <t>P4HB</t>
+  </si>
+  <si>
+    <t>ERO1A</t>
+  </si>
+  <si>
+    <t>ERO1B</t>
+  </si>
+  <si>
+    <t>ENSG00000185624</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000185624</t>
+  </si>
+  <si>
+    <t>ENSG00000197930</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000197930</t>
+  </si>
+  <si>
+    <t>ENSG00000086619</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000086619</t>
+  </si>
+  <si>
+    <t>PREB</t>
+  </si>
+  <si>
+    <t>SAR1A</t>
+  </si>
+  <si>
+    <t>SAR1B</t>
+  </si>
+  <si>
+    <t>SEC23A</t>
+  </si>
+  <si>
+    <t>SEC23B</t>
+  </si>
+  <si>
+    <t>SEC24A</t>
+  </si>
+  <si>
+    <t>SEC24B</t>
+  </si>
+  <si>
+    <t>SEC24C</t>
+  </si>
+  <si>
+    <t>SEC24D</t>
+  </si>
+  <si>
+    <t>ENSG00000138073</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000138073</t>
+  </si>
+  <si>
+    <t>ENSG00000079332</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000079332</t>
+  </si>
+  <si>
+    <t>ENSG00000152700</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000152700</t>
+  </si>
+  <si>
+    <t>ENSG00000100934</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000100934</t>
+  </si>
+  <si>
+    <t>ENSG00000101310</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000101310</t>
+  </si>
+  <si>
+    <t>ENSG00000113615</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000113615</t>
+  </si>
+  <si>
+    <t>ENSG00000138802</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000138802</t>
+  </si>
+  <si>
+    <t>ENSG00000176986</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000176986</t>
+  </si>
+  <si>
+    <t>ENSG00000150961</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000150961</t>
+  </si>
+  <si>
+    <t>SEC13</t>
+  </si>
+  <si>
+    <t>SEC31A</t>
+  </si>
+  <si>
+    <t>SEC31B</t>
+  </si>
+  <si>
+    <t>ENSG00000157020</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000157020</t>
+  </si>
+  <si>
+    <t>ENSG00000138674</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000138674</t>
+  </si>
+  <si>
+    <t>ENSG00000075826</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000075826</t>
+  </si>
+  <si>
+    <t>ENSG00000175582</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000175582</t>
+  </si>
+  <si>
+    <t>RAB6A</t>
+  </si>
+  <si>
+    <t>ENST00000310653</t>
+  </si>
+  <si>
+    <t>ensemble/ENST00000310653</t>
+  </si>
+  <si>
+    <t>RAB6A1</t>
+  </si>
+  <si>
+    <t>GOLGA4</t>
+  </si>
+  <si>
+    <t>ENSG00000144674</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000144674</t>
+  </si>
+  <si>
+    <t>RAB6B</t>
+  </si>
+  <si>
+    <t>ENSG00000154917</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000154917</t>
+  </si>
+  <si>
+    <t>PIK3CD</t>
+  </si>
+  <si>
+    <t>ENSG00000171608</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000171608</t>
+  </si>
+  <si>
+    <t>STX4</t>
+  </si>
+  <si>
+    <t>STX6</t>
+  </si>
+  <si>
+    <t>STX7</t>
+  </si>
+  <si>
+    <t>VTI1B</t>
+  </si>
+  <si>
+    <t>VAMP3</t>
+  </si>
+  <si>
+    <t>SNAP23</t>
+  </si>
+  <si>
+    <t>ENSG00000103496</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000103496</t>
+  </si>
+  <si>
+    <t>ENSG00000135823</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000135823</t>
+  </si>
+  <si>
+    <t>ENSG00000079950</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000079950</t>
+  </si>
+  <si>
+    <t>ENSG00000100568</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000100568</t>
+  </si>
+  <si>
+    <t>ENSG00000049245</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000049245</t>
+  </si>
+  <si>
+    <t>ENSG00000092531</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000092531</t>
+  </si>
+  <si>
+    <t>RHBDF2</t>
+  </si>
+  <si>
+    <t>FURIN</t>
+  </si>
+  <si>
+    <t>ADAM17</t>
+  </si>
+  <si>
+    <t>FRMD8</t>
+  </si>
+  <si>
+    <t>PCSK7</t>
+  </si>
+  <si>
+    <t>ENSG00000129667</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000129667</t>
+  </si>
+  <si>
+    <t>ENSG00000140564</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000140564</t>
+  </si>
+  <si>
+    <t>ENSG00000151694</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000151694</t>
+  </si>
+  <si>
+    <t>ENSG00000126391</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000126391</t>
+  </si>
+  <si>
+    <t>ENSG00000160613</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000160613</t>
+  </si>
+  <si>
+    <t>TNFRSF1A</t>
+  </si>
+  <si>
+    <t>TNFRSF1B</t>
+  </si>
+  <si>
+    <t>ENSG00000067182</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000067182</t>
+  </si>
+  <si>
+    <t>ENSG00000028137</t>
+  </si>
+  <si>
+    <t>ensemble/ENSG00000028137</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -64,6 +517,11 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow (Body)"/>
     </font>
   </fonts>
   <fills count="2">
@@ -86,9 +544,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -423,14 +882,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1C1BC65-DA0E-44C0-A004-5AEFCAAD595E}">
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <dimension ref="A1:C52"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="17.875" customWidth="1"/>
-    <col min="2" max="2" width="22.125" customWidth="1"/>
+    <col min="1" max="1" width="17.83203125" customWidth="1"/>
+    <col min="2" max="2" width="22.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -439,6 +898,567 @@
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>45</v>
+      </c>
+      <c r="B15" t="s">
+        <v>46</v>
+      </c>
+      <c r="C15" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" t="s">
+        <v>48</v>
+      </c>
+      <c r="C16" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B17" t="s">
+        <v>50</v>
+      </c>
+      <c r="C17" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>51</v>
+      </c>
+      <c r="B18" t="s">
+        <v>52</v>
+      </c>
+      <c r="C18" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>53</v>
+      </c>
+      <c r="B19" t="s">
+        <v>54</v>
+      </c>
+      <c r="C19" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B20" t="s">
+        <v>59</v>
+      </c>
+      <c r="C20" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>60</v>
+      </c>
+      <c r="B21" t="s">
+        <v>61</v>
+      </c>
+      <c r="C21" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C22" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>73</v>
+      </c>
+      <c r="B23" t="s">
+        <v>74</v>
+      </c>
+      <c r="C23" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>75</v>
+      </c>
+      <c r="B24" t="s">
+        <v>76</v>
+      </c>
+      <c r="C24" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>77</v>
+      </c>
+      <c r="B25" t="s">
+        <v>78</v>
+      </c>
+      <c r="C25" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>79</v>
+      </c>
+      <c r="B26" t="s">
+        <v>80</v>
+      </c>
+      <c r="C26" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>81</v>
+      </c>
+      <c r="B27" t="s">
+        <v>82</v>
+      </c>
+      <c r="C27" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>83</v>
+      </c>
+      <c r="B28" t="s">
+        <v>84</v>
+      </c>
+      <c r="C28" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>85</v>
+      </c>
+      <c r="B29" t="s">
+        <v>86</v>
+      </c>
+      <c r="C29" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>87</v>
+      </c>
+      <c r="B30" t="s">
+        <v>88</v>
+      </c>
+      <c r="C30" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>89</v>
+      </c>
+      <c r="B31" t="s">
+        <v>90</v>
+      </c>
+      <c r="C31" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>94</v>
+      </c>
+      <c r="B32" t="s">
+        <v>95</v>
+      </c>
+      <c r="C32" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>96</v>
+      </c>
+      <c r="B33" t="s">
+        <v>97</v>
+      </c>
+      <c r="C33" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>98</v>
+      </c>
+      <c r="B34" t="s">
+        <v>99</v>
+      </c>
+      <c r="C34" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>107</v>
+      </c>
+      <c r="B35" t="s">
+        <v>108</v>
+      </c>
+      <c r="C35" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>100</v>
+      </c>
+      <c r="B36" t="s">
+        <v>101</v>
+      </c>
+      <c r="C36" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>103</v>
+      </c>
+      <c r="B37" t="s">
+        <v>104</v>
+      </c>
+      <c r="C37" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>110</v>
+      </c>
+      <c r="B38" t="s">
+        <v>111</v>
+      </c>
+      <c r="C38" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>113</v>
+      </c>
+      <c r="B39" t="s">
+        <v>114</v>
+      </c>
+      <c r="C39" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>121</v>
+      </c>
+      <c r="B40" t="s">
+        <v>122</v>
+      </c>
+      <c r="C40" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>123</v>
+      </c>
+      <c r="B41" t="s">
+        <v>124</v>
+      </c>
+      <c r="C41" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>125</v>
+      </c>
+      <c r="B42" t="s">
+        <v>126</v>
+      </c>
+      <c r="C42" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>127</v>
+      </c>
+      <c r="B43" t="s">
+        <v>128</v>
+      </c>
+      <c r="C43" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>129</v>
+      </c>
+      <c r="B44" t="s">
+        <v>130</v>
+      </c>
+      <c r="C44" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>131</v>
+      </c>
+      <c r="B45" t="s">
+        <v>132</v>
+      </c>
+      <c r="C45" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>138</v>
+      </c>
+      <c r="B46" t="s">
+        <v>139</v>
+      </c>
+      <c r="C46" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>140</v>
+      </c>
+      <c r="B47" t="s">
+        <v>141</v>
+      </c>
+      <c r="C47" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>142</v>
+      </c>
+      <c r="B48" t="s">
+        <v>143</v>
+      </c>
+      <c r="C48" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>144</v>
+      </c>
+      <c r="B49" t="s">
+        <v>145</v>
+      </c>
+      <c r="C49" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>146</v>
+      </c>
+      <c r="B50" t="s">
+        <v>147</v>
+      </c>
+      <c r="C50" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>150</v>
+      </c>
+      <c r="B51" t="s">
+        <v>151</v>
+      </c>
+      <c r="C51" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>152</v>
+      </c>
+      <c r="B52" t="s">
+        <v>153</v>
+      </c>
+      <c r="C52" t="s">
+        <v>149</v>
       </c>
     </row>
   </sheetData>

</xml_diff>